<commit_message>
clean up| all finish
</commit_message>
<xml_diff>
--- a/5/search/FY2_Missile1_results/all_solutions.xlsx
+++ b/5/search/FY2_Missile1_results/all_solutions.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K18"/>
+  <dimension ref="A1:K31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -487,597 +487,1052 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>225</v>
+        <v>211.5</v>
       </c>
       <c r="B2" t="n">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="C2" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="D2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E2" t="n">
-        <v>11168.44242532462</v>
+        <v>10553.92228125546</v>
       </c>
       <c r="F2" t="n">
-        <v>568.4424253246202</v>
+        <v>513.842434241751</v>
       </c>
       <c r="G2" t="n">
         <v>1400</v>
       </c>
       <c r="H2" t="n">
-        <v>10614.07070887437</v>
+        <v>9740.503564461656</v>
       </c>
       <c r="I2" t="n">
-        <v>14.07070887436703</v>
+        <v>15.37880350273593</v>
       </c>
       <c r="J2" t="n">
-        <v>1086.4</v>
+        <v>1003.1</v>
       </c>
       <c r="K2" t="n">
-        <v>3.300000000000001</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>225</v>
+        <v>211.5</v>
       </c>
       <c r="B3" t="n">
-        <v>120.4</v>
+        <v>124</v>
       </c>
       <c r="C3" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D3" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E3" t="n">
-        <v>11318.91474836112</v>
+        <v>10731.27143544111</v>
       </c>
       <c r="F3" t="n">
-        <v>718.9147483611174</v>
+        <v>622.5221357026684</v>
       </c>
       <c r="G3" t="n">
         <v>1400</v>
       </c>
       <c r="H3" t="n">
-        <v>10637.82949672224</v>
+        <v>9779.725012021943</v>
       </c>
       <c r="I3" t="n">
-        <v>37.82949672223481</v>
+        <v>39.41373747966963</v>
       </c>
       <c r="J3" t="n">
-        <v>1086.4</v>
+        <v>1003.1</v>
       </c>
       <c r="K3" t="n">
-        <v>3.600000000000001</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>243</v>
+        <v>211.5</v>
       </c>
       <c r="B4" t="n">
-        <v>103.6</v>
+        <v>126</v>
       </c>
       <c r="C4" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E4" t="n">
-        <v>11623.73267381586</v>
+        <v>10710.80807149661</v>
       </c>
       <c r="F4" t="n">
-        <v>661.5337927526808</v>
+        <v>609.9821701494855</v>
       </c>
       <c r="G4" t="n">
         <v>1400</v>
       </c>
       <c r="H4" t="n">
-        <v>11294.49876340474</v>
+        <v>9743.914125119072</v>
       </c>
       <c r="I4" t="n">
-        <v>15.37586141127656</v>
+        <v>17.4687977615996</v>
       </c>
       <c r="J4" t="n">
-        <v>1159.9</v>
+        <v>1003.1</v>
       </c>
       <c r="K4" t="n">
-        <v>3.400000000000002</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>243</v>
+        <v>220.5</v>
       </c>
       <c r="B5" t="n">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="C5" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E5" t="n">
-        <v>11745.76532014585</v>
+        <v>11184.84480487677</v>
       </c>
       <c r="F5" t="n">
-        <v>901.036346454514</v>
+        <v>703.7916921900432</v>
       </c>
       <c r="G5" t="n">
         <v>1400</v>
       </c>
       <c r="H5" t="n">
-        <v>11300.8546304011</v>
+        <v>10369.68960975353</v>
       </c>
       <c r="I5" t="n">
-        <v>27.84995274991365</v>
+        <v>7.5833843800865</v>
       </c>
       <c r="J5" t="n">
-        <v>1159.9</v>
+        <v>1086.4</v>
       </c>
       <c r="K5" t="n">
-        <v>2.800000000000001</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>252</v>
+        <v>225</v>
       </c>
       <c r="B6" t="n">
-        <v>75.59999999999999</v>
+        <v>120</v>
       </c>
       <c r="C6" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="D6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E6" t="n">
-        <v>11719.65978270305</v>
+        <v>11321.17749006091</v>
       </c>
       <c r="F6" t="n">
-        <v>537.2015284170368</v>
+        <v>721.1774900609145</v>
       </c>
       <c r="G6" t="n">
         <v>1400</v>
       </c>
       <c r="H6" t="n">
-        <v>11556.12798927982</v>
+        <v>10642.35498012183</v>
       </c>
       <c r="I6" t="n">
-        <v>33.90241999364162</v>
+        <v>42.35498012182893</v>
       </c>
       <c r="J6" t="n">
-        <v>1159.9</v>
+        <v>1086.4</v>
       </c>
       <c r="K6" t="n">
-        <v>3.100000000000001</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>252</v>
+        <v>229.5</v>
       </c>
       <c r="B7" t="n">
-        <v>95.2</v>
+        <v>110</v>
       </c>
       <c r="C7" t="n">
         <v>8</v>
       </c>
       <c r="D7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E7" t="n">
-        <v>11764.65265708404</v>
+        <v>11428.48571746944</v>
       </c>
       <c r="F7" t="n">
-        <v>675.6753571896111</v>
+        <v>730.8427502719726</v>
       </c>
       <c r="G7" t="n">
         <v>1400</v>
       </c>
       <c r="H7" t="n">
-        <v>11558.72373203257</v>
+        <v>10856.97143493888</v>
       </c>
       <c r="I7" t="n">
-        <v>41.89129473052071</v>
+        <v>61.68550054394518</v>
       </c>
       <c r="J7" t="n">
-        <v>1159.9</v>
+        <v>1086.4</v>
       </c>
       <c r="K7" t="n">
-        <v>3.200000000000001</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>252</v>
+        <v>243</v>
       </c>
       <c r="B8" t="n">
-        <v>128.8</v>
+        <v>102</v>
       </c>
       <c r="C8" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D8" t="n">
         <v>7</v>
       </c>
       <c r="E8" t="n">
-        <v>11840.79444449803</v>
+        <v>11629.54375221253</v>
       </c>
       <c r="F8" t="n">
-        <v>910.0156828047368</v>
+        <v>672.9386762622919</v>
       </c>
       <c r="G8" t="n">
         <v>1400</v>
       </c>
       <c r="H8" t="n">
-        <v>11562.18472236957</v>
+        <v>11305.39453539849</v>
       </c>
       <c r="I8" t="n">
-        <v>52.54312771302625</v>
+        <v>36.76001799179733</v>
       </c>
       <c r="J8" t="n">
         <v>1159.9</v>
       </c>
       <c r="K8" t="n">
-        <v>2.4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>261</v>
+        <v>243</v>
       </c>
       <c r="B9" t="n">
-        <v>100.8</v>
+        <v>104</v>
       </c>
       <c r="C9" t="n">
         <v>8</v>
       </c>
       <c r="D9" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E9" t="n">
-        <v>11873.85124739156</v>
+        <v>11622.2799042167</v>
       </c>
       <c r="F9" t="n">
-        <v>603.5281221440811</v>
+        <v>658.682571875278</v>
       </c>
       <c r="G9" t="n">
         <v>1400</v>
       </c>
       <c r="H9" t="n">
-        <v>11779.23968293523</v>
+        <v>11291.77482040631</v>
       </c>
       <c r="I9" t="n">
-        <v>6.174213752141895</v>
+        <v>10.0298222661462</v>
       </c>
       <c r="J9" t="n">
-        <v>1223.6</v>
+        <v>1159.9</v>
       </c>
       <c r="K9" t="n">
-        <v>1.699999999999999</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>261</v>
+        <v>243</v>
       </c>
       <c r="B10" t="n">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C10" t="n">
         <v>4</v>
       </c>
       <c r="D10" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E10" t="n">
-        <v>11912.39669957747</v>
+        <v>11749.39724414377</v>
       </c>
       <c r="F10" t="n">
-        <v>846.8945292667229</v>
+        <v>908.164398648021</v>
       </c>
       <c r="G10" t="n">
         <v>1400</v>
       </c>
       <c r="H10" t="n">
-        <v>11780.99174894368</v>
+        <v>11310.84242139537</v>
       </c>
       <c r="I10" t="n">
-        <v>17.23632316680721</v>
+        <v>47.45209628205771</v>
       </c>
       <c r="J10" t="n">
-        <v>1223.6</v>
+        <v>1159.9</v>
       </c>
       <c r="K10" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>270</v>
+        <v>243</v>
       </c>
       <c r="B11" t="n">
-        <v>98</v>
+        <v>140</v>
       </c>
       <c r="C11" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D11" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E11" t="n">
-        <v>12000</v>
+        <v>11745.76532014585</v>
       </c>
       <c r="F11" t="n">
-        <v>616</v>
+        <v>901.036346454514</v>
       </c>
       <c r="G11" t="n">
         <v>1400</v>
       </c>
       <c r="H11" t="n">
-        <v>12000</v>
+        <v>11300.8546304011</v>
       </c>
       <c r="I11" t="n">
-        <v>28</v>
+        <v>27.84995274991365</v>
       </c>
       <c r="J11" t="n">
-        <v>1223.6</v>
+        <v>1159.9</v>
       </c>
       <c r="K11" t="n">
-        <v>3.600000000000001</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>270</v>
+        <v>247.5</v>
       </c>
       <c r="B12" t="n">
-        <v>137.2</v>
+        <v>132</v>
       </c>
       <c r="C12" t="n">
         <v>4</v>
       </c>
       <c r="D12" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E12" t="n">
-        <v>12000</v>
+        <v>11797.94314771123</v>
       </c>
       <c r="F12" t="n">
-        <v>851.2</v>
+        <v>912.1916068340406</v>
       </c>
       <c r="G12" t="n">
         <v>1400</v>
       </c>
       <c r="H12" t="n">
-        <v>12000</v>
+        <v>11444.34365620589</v>
       </c>
       <c r="I12" t="n">
-        <v>28.00000000000011</v>
+        <v>58.52691879361157</v>
       </c>
       <c r="J12" t="n">
-        <v>1223.6</v>
+        <v>1159.9</v>
       </c>
       <c r="K12" t="n">
-        <v>2.599999999999998</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>279</v>
+        <v>252</v>
       </c>
       <c r="B13" t="n">
-        <v>98</v>
+        <v>128</v>
       </c>
       <c r="C13" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D13" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E13" t="n">
-        <v>12122.64462059154</v>
+        <v>11841.78329888003</v>
       </c>
       <c r="F13" t="n">
-        <v>625.652340973412</v>
+        <v>913.0590636568813</v>
       </c>
       <c r="G13" t="n">
         <v>1400</v>
       </c>
       <c r="H13" t="n">
-        <v>12214.6280860352</v>
+        <v>11564.90407192007</v>
       </c>
       <c r="I13" t="n">
-        <v>44.89159670347112</v>
+        <v>60.91242505642379</v>
       </c>
       <c r="J13" t="n">
-        <v>1223.6</v>
+        <v>1159.9</v>
       </c>
       <c r="K13" t="n">
-        <v>2.199999999999999</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>288</v>
+        <v>261</v>
       </c>
       <c r="B14" t="n">
-        <v>86.8</v>
+        <v>140</v>
       </c>
       <c r="C14" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="D14" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E14" t="n">
-        <v>12321.87210134094</v>
+        <v>11912.39669957747</v>
       </c>
       <c r="F14" t="n">
-        <v>409.3795326269681</v>
+        <v>846.8945292667229</v>
       </c>
       <c r="G14" t="n">
         <v>1400</v>
       </c>
       <c r="H14" t="n">
-        <v>12455.98547689967</v>
+        <v>11780.99174894368</v>
       </c>
       <c r="I14" t="n">
-        <v>-3.378995445128623</v>
+        <v>17.23632316680721</v>
       </c>
       <c r="J14" t="n">
-        <v>1277.5</v>
+        <v>1223.6</v>
       </c>
       <c r="K14" t="n">
-        <v>0.3999999999999986</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>288</v>
+        <v>265.5</v>
       </c>
       <c r="B15" t="n">
-        <v>112</v>
+        <v>100</v>
       </c>
       <c r="C15" t="n">
         <v>8</v>
       </c>
       <c r="D15" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E15" t="n">
-        <v>12276.87922695995</v>
+        <v>11937.23272341772</v>
       </c>
       <c r="F15" t="n">
-        <v>547.8533613995423</v>
+        <v>602.4661330134976</v>
       </c>
       <c r="G15" t="n">
         <v>1400</v>
       </c>
       <c r="H15" t="n">
-        <v>12449.92874380992</v>
+        <v>11890.15726598102</v>
       </c>
       <c r="I15" t="n">
-        <v>15.2617122742563</v>
+        <v>4.315732773620766</v>
       </c>
       <c r="J15" t="n">
-        <v>1277.5</v>
+        <v>1223.6</v>
       </c>
       <c r="K15" t="n">
-        <v>3.400000000000002</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>297</v>
+        <v>265.5</v>
       </c>
       <c r="B16" t="n">
-        <v>117.6</v>
+        <v>138</v>
       </c>
       <c r="C16" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D16" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E16" t="n">
-        <v>12427.11426215497</v>
+        <v>11956.69057915823</v>
       </c>
       <c r="F16" t="n">
-        <v>561.7410620435834</v>
+        <v>849.7016317793134</v>
       </c>
       <c r="G16" t="n">
         <v>1400</v>
       </c>
       <c r="H16" t="n">
-        <v>12694.06067600182</v>
+        <v>11891.72644789557</v>
       </c>
       <c r="I16" t="n">
-        <v>37.82922582082301</v>
+        <v>24.25407944828351</v>
       </c>
       <c r="J16" t="n">
-        <v>1277.5</v>
+        <v>1223.6</v>
       </c>
       <c r="K16" t="n">
-        <v>3.800000000000001</v>
+        <v>4</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>315</v>
+        <v>270</v>
       </c>
       <c r="B17" t="n">
-        <v>131.6</v>
+        <v>136</v>
       </c>
       <c r="C17" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="D17" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E17" t="n">
-        <v>13116.66302884979</v>
+        <v>12000</v>
       </c>
       <c r="F17" t="n">
-        <v>283.3369711502039</v>
+        <v>856</v>
       </c>
       <c r="G17" t="n">
         <v>1400</v>
       </c>
       <c r="H17" t="n">
-        <v>13395.82878606224</v>
+        <v>12000</v>
       </c>
       <c r="I17" t="n">
-        <v>4.171213937754885</v>
+        <v>40</v>
       </c>
       <c r="J17" t="n">
-        <v>1355.9</v>
+        <v>1223.6</v>
       </c>
       <c r="K17" t="n">
-        <v>3.100000000000001</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
+        <v>274.5</v>
+      </c>
+      <c r="B18" t="n">
+        <v>136</v>
+      </c>
+      <c r="C18" t="n">
+        <v>4</v>
+      </c>
+      <c r="D18" t="n">
+        <v>6</v>
+      </c>
+      <c r="E18" t="n">
+        <v>12042.68174807595</v>
+      </c>
+      <c r="F18" t="n">
+        <v>857.6769704491784</v>
+      </c>
+      <c r="G18" t="n">
+        <v>1400</v>
+      </c>
+      <c r="H18" t="n">
+        <v>12106.70437018987</v>
+      </c>
+      <c r="I18" t="n">
+        <v>44.1924261229459</v>
+      </c>
+      <c r="J18" t="n">
+        <v>1223.6</v>
+      </c>
+      <c r="K18" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>279</v>
+      </c>
+      <c r="B19" t="n">
+        <v>136</v>
+      </c>
+      <c r="C19" t="n">
+        <v>4</v>
+      </c>
+      <c r="D19" t="n">
+        <v>6</v>
+      </c>
+      <c r="E19" t="n">
+        <v>12085.10034898188</v>
+      </c>
+      <c r="F19" t="n">
+        <v>862.697542716245</v>
+      </c>
+      <c r="G19" t="n">
+        <v>1400</v>
+      </c>
+      <c r="H19" t="n">
+        <v>12212.75087245471</v>
+      </c>
+      <c r="I19" t="n">
+        <v>56.74385679061254</v>
+      </c>
+      <c r="J19" t="n">
+        <v>1223.6</v>
+      </c>
+      <c r="K19" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>288</v>
+      </c>
+      <c r="B20" t="n">
+        <v>112</v>
+      </c>
+      <c r="C20" t="n">
+        <v>8</v>
+      </c>
+      <c r="D20" t="n">
+        <v>5</v>
+      </c>
+      <c r="E20" t="n">
+        <v>12276.87922695995</v>
+      </c>
+      <c r="F20" t="n">
+        <v>547.8533613995423</v>
+      </c>
+      <c r="G20" t="n">
+        <v>1400</v>
+      </c>
+      <c r="H20" t="n">
+        <v>12449.92874380992</v>
+      </c>
+      <c r="I20" t="n">
+        <v>15.2617122742563</v>
+      </c>
+      <c r="J20" t="n">
+        <v>1277.5</v>
+      </c>
+      <c r="K20" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>292.5</v>
+      </c>
+      <c r="B21" t="n">
+        <v>114</v>
+      </c>
+      <c r="C21" t="n">
+        <v>8</v>
+      </c>
+      <c r="D21" t="n">
+        <v>5</v>
+      </c>
+      <c r="E21" t="n">
+        <v>12349.00729031696</v>
+      </c>
+      <c r="F21" t="n">
+        <v>557.4218663497066</v>
+      </c>
+      <c r="G21" t="n">
+        <v>1400</v>
+      </c>
+      <c r="H21" t="n">
+        <v>12567.13684676506</v>
+      </c>
+      <c r="I21" t="n">
+        <v>30.81053281827326</v>
+      </c>
+      <c r="J21" t="n">
+        <v>1277.5</v>
+      </c>
+      <c r="K21" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>297</v>
+      </c>
+      <c r="B22" t="n">
+        <v>118</v>
+      </c>
+      <c r="C22" t="n">
+        <v>8</v>
+      </c>
+      <c r="D22" t="n">
+        <v>5</v>
+      </c>
+      <c r="E22" t="n">
+        <v>12428.56703175413</v>
+      </c>
+      <c r="F22" t="n">
+        <v>558.8898411661806</v>
+      </c>
+      <c r="G22" t="n">
+        <v>1400</v>
+      </c>
+      <c r="H22" t="n">
+        <v>12696.42142660046</v>
+      </c>
+      <c r="I22" t="n">
+        <v>33.19599189504356</v>
+      </c>
+      <c r="J22" t="n">
+        <v>1277.5</v>
+      </c>
+      <c r="K22" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>301.5</v>
+      </c>
+      <c r="B23" t="n">
+        <v>136</v>
+      </c>
+      <c r="C23" t="n">
+        <v>8</v>
+      </c>
+      <c r="D23" t="n">
+        <v>4</v>
+      </c>
+      <c r="E23" t="n">
+        <v>12568.47843841095</v>
+      </c>
+      <c r="F23" t="n">
+        <v>472.3275011827478</v>
+      </c>
+      <c r="G23" t="n">
+        <v>1400</v>
+      </c>
+      <c r="H23" t="n">
+        <v>12852.71765761643</v>
+      </c>
+      <c r="I23" t="n">
+        <v>8.491251774121736</v>
+      </c>
+      <c r="J23" t="n">
+        <v>1321.6</v>
+      </c>
+      <c r="K23" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>306</v>
+      </c>
+      <c r="B24" t="n">
+        <v>108</v>
+      </c>
+      <c r="C24" t="n">
+        <v>12</v>
+      </c>
+      <c r="D24" t="n">
+        <v>4</v>
+      </c>
+      <c r="E24" t="n">
+        <v>12761.76968697105</v>
+      </c>
+      <c r="F24" t="n">
+        <v>351.5139752900679</v>
+      </c>
+      <c r="G24" t="n">
+        <v>1400</v>
+      </c>
+      <c r="H24" t="n">
+        <v>13015.69291596139</v>
+      </c>
+      <c r="I24" t="n">
+        <v>2.018633720090577</v>
+      </c>
+      <c r="J24" t="n">
+        <v>1321.6</v>
+      </c>
+      <c r="K24" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>310.5</v>
+      </c>
+      <c r="B25" t="n">
+        <v>114</v>
+      </c>
+      <c r="C25" t="n">
+        <v>12</v>
+      </c>
+      <c r="D25" t="n">
+        <v>4</v>
+      </c>
+      <c r="E25" t="n">
+        <v>12888.44493011569</v>
+      </c>
+      <c r="F25" t="n">
+        <v>359.7646390591578</v>
+      </c>
+      <c r="G25" t="n">
+        <v>1400</v>
+      </c>
+      <c r="H25" t="n">
+        <v>13184.59324015425</v>
+      </c>
+      <c r="I25" t="n">
+        <v>13.01951874554379</v>
+      </c>
+      <c r="J25" t="n">
+        <v>1321.6</v>
+      </c>
+      <c r="K25" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>315</v>
+      </c>
+      <c r="B26" t="n">
+        <v>104</v>
+      </c>
+      <c r="C26" t="n">
+        <v>16</v>
+      </c>
+      <c r="D26" t="n">
+        <v>3</v>
+      </c>
+      <c r="E26" t="n">
+        <v>13176.62568389442</v>
+      </c>
+      <c r="F26" t="n">
+        <v>223.3743161055847</v>
+      </c>
+      <c r="G26" t="n">
+        <v>1400</v>
+      </c>
+      <c r="H26" t="n">
+        <v>13397.24299962462</v>
+      </c>
+      <c r="I26" t="n">
+        <v>2.757000375381892</v>
+      </c>
+      <c r="J26" t="n">
+        <v>1355.9</v>
+      </c>
+      <c r="K26" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>315</v>
+      </c>
+      <c r="B27" t="n">
+        <v>130</v>
+      </c>
+      <c r="C27" t="n">
+        <v>12</v>
+      </c>
+      <c r="D27" t="n">
+        <v>3</v>
+      </c>
+      <c r="E27" t="n">
+        <v>13103.08657865101</v>
+      </c>
+      <c r="F27" t="n">
+        <v>296.9134213489856</v>
+      </c>
+      <c r="G27" t="n">
+        <v>1400</v>
+      </c>
+      <c r="H27" t="n">
+        <v>13378.85822331377</v>
+      </c>
+      <c r="I27" t="n">
+        <v>21.14177668623199</v>
+      </c>
+      <c r="J27" t="n">
+        <v>1355.9</v>
+      </c>
+      <c r="K27" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>315</v>
+      </c>
+      <c r="B28" t="n">
+        <v>132</v>
+      </c>
+      <c r="C28" t="n">
+        <v>12</v>
+      </c>
+      <c r="D28" t="n">
+        <v>3</v>
+      </c>
+      <c r="E28" t="n">
+        <v>13120.05714139949</v>
+      </c>
+      <c r="F28" t="n">
+        <v>279.9428586005085</v>
+      </c>
+      <c r="G28" t="n">
+        <v>1400</v>
+      </c>
+      <c r="H28" t="n">
+        <v>13400.07142674936</v>
+      </c>
+      <c r="I28" t="n">
+        <v>-0.07142674936432059</v>
+      </c>
+      <c r="J28" t="n">
+        <v>1355.9</v>
+      </c>
+      <c r="K28" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>319.5</v>
+      </c>
+      <c r="B29" t="n">
+        <v>120</v>
+      </c>
+      <c r="C29" t="n">
+        <v>16</v>
+      </c>
+      <c r="D29" t="n">
+        <v>2</v>
+      </c>
+      <c r="E29" t="n">
+        <v>13459.97945395206</v>
+      </c>
+      <c r="F29" t="n">
+        <v>153.0597472060479</v>
+      </c>
+      <c r="G29" t="n">
+        <v>1400</v>
+      </c>
+      <c r="H29" t="n">
+        <v>13642.47688569607</v>
+      </c>
+      <c r="I29" t="n">
+        <v>-2.807784393196158</v>
+      </c>
+      <c r="J29" t="n">
+        <v>1380.4</v>
+      </c>
+      <c r="K29" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
         <v>324</v>
       </c>
-      <c r="B18" t="n">
+      <c r="B30" t="n">
+        <v>138</v>
+      </c>
+      <c r="C30" t="n">
+        <v>16</v>
+      </c>
+      <c r="D30" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" t="n">
+        <v>13786.30952357988</v>
+      </c>
+      <c r="F30" t="n">
+        <v>102.1701629382187</v>
+      </c>
+      <c r="G30" t="n">
+        <v>1400</v>
+      </c>
+      <c r="H30" t="n">
+        <v>13897.95386880363</v>
+      </c>
+      <c r="I30" t="n">
+        <v>21.05579812185738</v>
+      </c>
+      <c r="J30" t="n">
+        <v>1395.1</v>
+      </c>
+      <c r="K30" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>324</v>
+      </c>
+      <c r="B31" t="n">
         <v>140</v>
       </c>
-      <c r="C18" t="n">
+      <c r="C31" t="n">
         <v>16</v>
       </c>
-      <c r="D18" t="n">
+      <c r="D31" t="n">
         <v>1</v>
       </c>
-      <c r="E18" t="n">
+      <c r="E31" t="n">
         <v>13812.19806739988</v>
       </c>
-      <c r="F18" t="n">
+      <c r="F31" t="n">
         <v>83.36103486485968</v>
       </c>
-      <c r="G18" t="n">
-        <v>1400</v>
-      </c>
-      <c r="H18" t="n">
+      <c r="G31" t="n">
+        <v>1400</v>
+      </c>
+      <c r="H31" t="n">
         <v>13925.46044661237</v>
       </c>
-      <c r="I18" t="n">
+      <c r="I31" t="n">
         <v>1.071099543913405</v>
       </c>
-      <c r="J18" t="n">
+      <c r="J31" t="n">
         <v>1395.1</v>
       </c>
-      <c r="K18" t="n">
-        <v>2.600000000000001</v>
+      <c r="K31" t="n">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>